<commit_message>
docs: add project reference manual info.md, update dashboard layout and remove triangulation matrix, update test inputs
</commit_message>
<xml_diff>
--- a/data/audit_sheet.xlsx
+++ b/data/audit_sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,16 @@
           <t>agreement</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>new_sharpened_theme</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>new_agreement</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,6 +499,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +546,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,6 +593,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -600,6 +640,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ux_friction</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +687,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>delivery_ops</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -674,6 +734,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>habit_loop</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,6 +781,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -748,6 +828,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -785,6 +875,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>mental_model</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -822,6 +922,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -859,6 +969,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -896,6 +1016,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>delivery_ops</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -933,6 +1063,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -970,6 +1110,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1007,6 +1157,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1044,6 +1204,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1081,6 +1251,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ux_friction</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1118,6 +1298,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1155,6 +1345,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1192,6 +1392,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1229,6 +1439,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>delivery_ops</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1266,6 +1486,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1303,6 +1533,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1340,6 +1580,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>price_value</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1377,6 +1627,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1414,6 +1674,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1451,6 +1721,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1488,6 +1768,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1525,6 +1815,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>delivery_ops</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1562,6 +1862,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1599,6 +1909,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>assortment_gap</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1636,6 +1956,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1673,6 +2003,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1710,6 +2050,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>delivery_ops</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1747,6 +2097,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1784,6 +2144,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1821,6 +2191,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>mental_model</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1858,6 +2238,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1895,6 +2285,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1932,6 +2332,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1969,6 +2379,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2006,6 +2426,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2043,6 +2473,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>trust_quality</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2080,6 +2520,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2117,6 +2567,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2154,6 +2614,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>ux_friction</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2191,6 +2661,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>ux_friction</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2228,6 +2708,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2265,6 +2755,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>emotional</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2298,6 +2798,16 @@
         </is>
       </c>
       <c r="G51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
style: refine dashboard header layout, typography spacing, illustration scaling, and badge styling
</commit_message>
<xml_diff>
--- a/data/audit_sheet.xlsx
+++ b/data/audit_sheet.xlsx
@@ -491,22 +491,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>ux_friction</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>price_value</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>price_value</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -580,12 +580,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -627,17 +627,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -768,12 +768,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>mental_model</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -956,12 +956,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>price_value</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1003,27 +1003,27 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>trust_quality</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1159,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>price_value</t>
+          <t>assortment_gap</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>trust_information</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1285,12 +1285,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1379,17 +1379,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>trust_quality</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>price_value</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1614,27 +1614,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1661,27 +1661,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>mental_model</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1708,27 +1708,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1817,12 +1817,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1849,12 +1849,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1943,12 +1943,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2131,12 +2131,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>trust_information</t>
+          <t>trust_quality</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>mental_model</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2277,22 +2277,22 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>assortment_gap</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>assortment_gap</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2522,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>trust_quality</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2601,12 +2601,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>delivery_ops</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2710,12 +2710,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>price_value</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2757,12 +2757,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>price_value</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">

</xml_diff>

<commit_message>
refactor: reorganize file structure to data/ and src/, and update triangulation survey to n=50 respondents
</commit_message>
<xml_diff>
--- a/data/audit_sheet.xlsx
+++ b/data/audit_sheet.xlsx
@@ -501,12 +501,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>price_value</t>
+          <t>ux_friction</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1629,12 +1629,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1723,12 +1723,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>habit_loop</t>
+          <t>emotional</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>ux_friction</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ux_friction</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2193,12 +2193,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2287,12 +2287,12 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>assortment_gap</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ux_friction</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2522,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>trust_quality</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>emotional</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2616,12 +2616,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>ux_friction</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>ux_friction</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2710,12 +2710,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>price_value</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2757,12 +2757,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>price_value</t>
+          <t>habit_loop</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>